<commit_message>
Upload fix ex and new jobs
</commit_message>
<xml_diff>
--- a/M2_Statistica_&_Excel/W3_D1.xlsx
+++ b/M2_Statistica_&_Excel/W3_D1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SZN\Desktop\EPICODE CORSO\esercizi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SZN\Desktop\EPICODE CORSO\esercizi\esercizi consegnati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7340BC45-4D8D-43EF-8A12-2D2CBD097558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF01F090-C713-46BD-BC5D-559EB8C577CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{A8D91010-E5B0-48E5-800B-00E95F259AB9}"/>
+    <workbookView xWindow="3720" yWindow="2520" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="2" xr2:uid="{A8D91010-E5B0-48E5-800B-00E95F259AB9}"/>
   </bookViews>
   <sheets>
     <sheet name="Assoluti_IVA" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="713">
   <si>
     <t>MONITOR</t>
   </si>
@@ -2203,6 +2203,15 @@
   </si>
   <si>
     <t>Tot_importo</t>
+  </si>
+  <si>
+    <t>tot_importo_fatture</t>
+  </si>
+  <si>
+    <t>Imoporto fattura &gt;40k</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -2216,7 +2225,7 @@
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2299,6 +2308,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -2350,7 +2365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -2469,11 +2484,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2595,9 +2619,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2607,13 +2628,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2634,20 +2652,11 @@
     <xf numFmtId="165" fontId="10" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2670,266 +2679,34 @@
     <xf numFmtId="167" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="49">
     <dxf>
       <font>
         <b val="0"/>
@@ -3029,6 +2806,71 @@
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -3082,13 +2924,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -3124,6 +2959,13 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -3156,6 +2998,385 @@
         </right>
         <top/>
         <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -3366,102 +3587,29 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -3470,50 +3618,6 @@
         </right>
         <top/>
         <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -3543,9 +3647,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Giudizio-style" pivot="0" count="3" xr9:uid="{2E52EE12-209A-47C2-8CDF-5D952512E77D}">
-      <tableStyleElement type="headerRow" dxfId="43"/>
-      <tableStyleElement type="firstRowStripe" dxfId="42"/>
-      <tableStyleElement type="secondRowStripe" dxfId="41"/>
+      <tableStyleElement type="headerRow" dxfId="48"/>
+      <tableStyleElement type="firstRowStripe" dxfId="47"/>
+      <tableStyleElement type="secondRowStripe" dxfId="46"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3560,59 +3664,59 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1CCF7C9-FAFB-4DA7-9D24-D726FF9ADD57}" name="Giudizio" displayName="Giudizio" ref="A1:D8" headerRowCount="0" headerRowDxfId="40" dataDxfId="39" totalsRowDxfId="37" tableBorderDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1CCF7C9-FAFB-4DA7-9D24-D726FF9ADD57}" name="Giudizio" displayName="Giudizio" ref="A1:D8" headerRowCount="0" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="17" tableBorderDxfId="18">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{74472EEE-8E39-4DAB-8BFC-2E5E835D3DD7}" name="Column1" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{F5B4876C-0C0B-47ED-B569-78D9E0EB393D}" name="Column2" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{2EFD64E9-403F-4A71-BA7A-2D5C38159F62}" name="Column3" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{B31FD795-8660-4D7C-A148-3D1F99ED2EB0}" name="Column4" headerRowDxfId="33" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{74472EEE-8E39-4DAB-8BFC-2E5E835D3DD7}" name="Column1" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{F5B4876C-0C0B-47ED-B569-78D9E0EB393D}" name="Column2" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{2EFD64E9-403F-4A71-BA7A-2D5C38159F62}" name="Column3" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{B31FD795-8660-4D7C-A148-3D1F99ED2EB0}" name="Column4" headerRowDxfId="13" dataDxfId="12" totalsRowDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="Giudizio-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{127BDB2C-14DA-4BB2-9F5F-E180FA1D8CAE}" name="Table2" displayName="Table2" ref="A1:E80" totalsRowShown="0" headerRowDxfId="10" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{127BDB2C-14DA-4BB2-9F5F-E180FA1D8CAE}" name="Table2" displayName="Table2" ref="A1:E80" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="41">
   <autoFilter ref="A1:E80" xr:uid="{127BDB2C-14DA-4BB2-9F5F-E180FA1D8CAE}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{14F89D16-B520-46BC-A082-6391E9B00EC5}" name="Data" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{D1A73F78-E3CC-4227-B2C2-71CD4693FE2E}" name="Cliente" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{45454885-5590-469D-A170-5E0BB8F46B87}" name="Categoria" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{2A061044-38E7-49EA-B874-7FB851E3442E}" name="Importo fattura" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{C1C9F864-EEE5-4B91-8DA9-E472D0810698}" name="Spese di spedizione" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{14F89D16-B520-46BC-A082-6391E9B00EC5}" name="Data" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{D1A73F78-E3CC-4227-B2C2-71CD4693FE2E}" name="Cliente" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{45454885-5590-469D-A170-5E0BB8F46B87}" name="Categoria" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{2A061044-38E7-49EA-B874-7FB851E3442E}" name="Importo fattura" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{C1C9F864-EEE5-4B91-8DA9-E472D0810698}" name="Spese di spedizione" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6557F6F2-A47A-4124-8331-0A4BCD661586}" name="fatture40k" displayName="fatture40k" ref="H47:L80" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6557F6F2-A47A-4124-8331-0A4BCD661586}" name="fatture40k" displayName="fatture40k" ref="H47:L81" totalsRowCount="1" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="H47:L80" xr:uid="{6557F6F2-A47A-4124-8331-0A4BCD661586}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{765D0489-1A46-4C80-802C-3FDCB9EE662D}" name="Data" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{AE3675DC-5678-406B-8D3D-28E1C75E162A}" name="Cliente" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{2A6210B9-6497-4C7C-A90F-2961CE5FF74C}" name="Categoria" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{73A4E6E0-5280-48A6-97D4-DE473FCB5159}" name="Importo fattura" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{FDB1BBF9-CD29-4908-8EE5-081D651F89E9}" name="Spese di spedizione" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{765D0489-1A46-4C80-802C-3FDCB9EE662D}" name="Data" totalsRowLabel="Total" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{AE3675DC-5678-406B-8D3D-28E1C75E162A}" name="Cliente" dataDxfId="28" totalsRowDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{2A6210B9-6497-4C7C-A90F-2961CE5FF74C}" name="Categoria" dataDxfId="26" totalsRowDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{73A4E6E0-5280-48A6-97D4-DE473FCB5159}" name="Importo fattura" totalsRowFunction="sum" dataDxfId="24" totalsRowDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{FDB1BBF9-CD29-4908-8EE5-081D651F89E9}" name="Spese di spedizione" totalsRowFunction="sum" dataDxfId="22" totalsRowDxfId="21"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C8CA392F-454A-4F55-BA31-E4A5F9DD17D5}" name="frutta" displayName="frutta" ref="A1:F47" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowBorderDxfId="18" tableBorderDxfId="19" totalsRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C8CA392F-454A-4F55-BA31-E4A5F9DD17D5}" name="frutta" displayName="frutta" ref="A1:F47" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:F47" xr:uid="{C8CA392F-454A-4F55-BA31-E4A5F9DD17D5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C3A66195-7D11-47D3-BEF0-07FDB51E90C5}" name="FRUTTA" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{D6D0A2FD-0B7A-4D3F-807A-1AC4F8778499}" name="PESO" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{FA8F424B-3461-4DDB-8383-43E40023D360}" name="COSTO OTTENUTO" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{C3A66195-7D11-47D3-BEF0-07FDB51E90C5}" name="FRUTTA" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{D6D0A2FD-0B7A-4D3F-807A-1AC4F8778499}" name="PESO" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{FA8F424B-3461-4DDB-8383-43E40023D360}" name="COSTO OTTENUTO" dataDxfId="3">
       <calculatedColumnFormula>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9EC8ADE3-A2F8-4157-B57B-9ADAD798C298}" name="COSTO" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{15F417E3-FAF7-4C88-B3F1-AB51181AE14C}" name="PREZZO UNITARIO " dataDxfId="13">
+    <tableColumn id="3" xr3:uid="{9EC8ADE3-A2F8-4157-B57B-9ADAD798C298}" name="COSTO" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{15F417E3-FAF7-4C88-B3F1-AB51181AE14C}" name="PREZZO UNITARIO " dataDxfId="1">
       <calculatedColumnFormula>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{750A75A2-828F-42B8-AA16-9D744C519FE2}" name="PREZZO UNITARIO MEDIO " dataDxfId="14">
+    <tableColumn id="8" xr3:uid="{750A75A2-828F-42B8-AA16-9D744C519FE2}" name="PREZZO UNITARIO MEDIO " dataDxfId="0">
       <calculatedColumnFormula>_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -33944,19 +34048,19 @@
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="54" t="s">
         <v>493</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="55" t="s">
         <v>494</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="55" t="s">
         <v>495</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="56" t="s">
         <v>496</v>
       </c>
-      <c r="E1" s="59" t="s">
+      <c r="E1" s="57" t="s">
         <v>497</v>
       </c>
       <c r="F1" s="6"/>
@@ -34010,7 +34114,7 @@
       <c r="E3" s="26">
         <v>29</v>
       </c>
-      <c r="H3" s="70" t="s">
+      <c r="H3" s="65" t="s">
         <v>495</v>
       </c>
       <c r="I3" s="11" t="s">
@@ -34033,7 +34137,7 @@
       <c r="E4" s="26">
         <v>21</v>
       </c>
-      <c r="H4" s="70" t="s">
+      <c r="H4" s="65" t="s">
         <v>584</v>
       </c>
       <c r="I4" s="11" cm="1">
@@ -34057,7 +34161,7 @@
       <c r="E5" s="26">
         <v>29</v>
       </c>
-      <c r="H5" s="70" t="s">
+      <c r="H5" s="65" t="s">
         <v>585</v>
       </c>
       <c r="I5" s="31">
@@ -34135,8 +34239,8 @@
       <c r="H9" s="10" t="s">
         <v>708</v>
       </c>
-      <c r="I9" s="47">
-        <v>40000</v>
+      <c r="I9" s="10" t="s">
+        <v>711</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34155,21 +34259,15 @@
       <c r="E10" s="26">
         <v>23</v>
       </c>
-      <c r="H10" s="63" t="s">
-        <v>493</v>
-      </c>
-      <c r="I10" s="63" t="s">
-        <v>494</v>
-      </c>
-      <c r="J10" s="63" t="s">
-        <v>495</v>
-      </c>
-      <c r="K10" s="64" t="s">
-        <v>496</v>
-      </c>
-      <c r="L10" s="64" t="s">
-        <v>497</v>
-      </c>
+      <c r="H10" s="68">
+        <v>40000</v>
+      </c>
+      <c r="I10" s="31" cm="1">
+        <f t="array" ref="I10:I42">_xlfn._xlws.SORT(_xlfn._xlws.FILTER(Table2[Importo fattura],Table2[Importo fattura]&gt;$H$10),1,-1)</f>
+        <v>2425000</v>
+      </c>
+      <c r="K10" s="70"/>
+      <c r="L10" s="70"/>
     </row>
     <row r="11" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="23">
@@ -34187,22 +34285,12 @@
       <c r="E11" s="26">
         <v>24</v>
       </c>
-      <c r="H11" s="60" cm="1">
-        <f t="array" ref="H11:L43">_xlfn._xlws.SORT(_xlfn._xlws.FILTER(Table2[],Table2[Importo fattura]&gt;=$I$9),4,-1)</f>
-        <v>36604</v>
-      </c>
-      <c r="I11" s="11" t="str">
-        <v>Gateway 2000</v>
-      </c>
-      <c r="J11" s="11" t="str">
-        <v>Hardware</v>
-      </c>
-      <c r="K11" s="31">
+      <c r="H11" s="72"/>
+      <c r="I11" s="73">
         <v>2425000</v>
       </c>
-      <c r="L11" s="11">
-        <v>11</v>
-      </c>
+      <c r="K11" s="71"/>
+      <c r="L11" s="71"/>
     </row>
     <row r="12" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="23">
@@ -34220,21 +34308,12 @@
       <c r="E12" s="26">
         <v>27</v>
       </c>
-      <c r="H12" s="60">
-        <v>36649</v>
-      </c>
-      <c r="I12" s="11" t="str">
-        <v>Gateway 2000</v>
-      </c>
-      <c r="J12" s="11" t="str">
-        <v>Hardware</v>
-      </c>
-      <c r="K12" s="31">
-        <v>2425000</v>
-      </c>
-      <c r="L12" s="11">
-        <v>21</v>
-      </c>
+      <c r="H12" s="72"/>
+      <c r="I12" s="31">
+        <v>1860000</v>
+      </c>
+      <c r="K12" s="71"/>
+      <c r="L12" s="71"/>
       <c r="M12" s="9"/>
     </row>
     <row r="13" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34253,21 +34332,12 @@
       <c r="E13" s="26">
         <v>15</v>
       </c>
-      <c r="H13" s="60">
-        <v>36651</v>
-      </c>
-      <c r="I13" s="11" t="str">
-        <v>Gateway 2000</v>
-      </c>
-      <c r="J13" s="11" t="str">
-        <v>Hardware</v>
-      </c>
-      <c r="K13" s="31">
-        <v>1860000</v>
-      </c>
-      <c r="L13" s="11">
-        <v>19</v>
-      </c>
+      <c r="H13" s="72"/>
+      <c r="I13" s="31">
+        <v>1368000</v>
+      </c>
+      <c r="K13" s="71"/>
+      <c r="L13" s="71"/>
       <c r="M13" s="9"/>
     </row>
     <row r="14" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34286,21 +34356,12 @@
       <c r="E14" s="26">
         <v>17</v>
       </c>
-      <c r="H14" s="60">
-        <v>36573</v>
-      </c>
-      <c r="I14" s="11" t="str">
-        <v>American Airlines</v>
-      </c>
-      <c r="J14" s="11" t="str">
-        <v>Viaggio d'affari</v>
-      </c>
-      <c r="K14" s="31">
-        <v>1368000</v>
-      </c>
-      <c r="L14" s="11">
-        <v>28</v>
-      </c>
+      <c r="H14" s="72"/>
+      <c r="I14" s="31">
+        <v>348980</v>
+      </c>
+      <c r="K14" s="71"/>
+      <c r="L14" s="71"/>
       <c r="M14" s="9"/>
     </row>
     <row r="15" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34319,21 +34380,12 @@
       <c r="E15" s="26">
         <v>13</v>
       </c>
-      <c r="H15" s="60">
-        <v>36555</v>
-      </c>
-      <c r="I15" s="11" t="str">
-        <v>Fletcher's for Children</v>
-      </c>
-      <c r="J15" s="11" t="str">
-        <v>Mobili</v>
-      </c>
-      <c r="K15" s="31">
-        <v>348980</v>
-      </c>
-      <c r="L15" s="11">
-        <v>15</v>
-      </c>
+      <c r="H15" s="72"/>
+      <c r="I15" s="31">
+        <v>295000</v>
+      </c>
+      <c r="K15" s="71"/>
+      <c r="L15" s="71"/>
       <c r="M15" s="9"/>
     </row>
     <row r="16" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34352,21 +34404,12 @@
       <c r="E16" s="26">
         <v>14</v>
       </c>
-      <c r="H16" s="60">
-        <v>36554</v>
-      </c>
-      <c r="I16" s="11" t="str">
-        <v>Agora Publishing</v>
-      </c>
-      <c r="J16" s="11" t="str">
-        <v>Manuali</v>
-      </c>
-      <c r="K16" s="31">
-        <v>295000</v>
-      </c>
-      <c r="L16" s="11">
-        <v>27</v>
-      </c>
+      <c r="H16" s="72"/>
+      <c r="I16" s="31">
+        <v>201000</v>
+      </c>
+      <c r="K16" s="71"/>
+      <c r="L16" s="71"/>
       <c r="M16" s="9"/>
     </row>
     <row r="17" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34385,21 +34428,12 @@
       <c r="E17" s="26">
         <v>28</v>
       </c>
-      <c r="H17" s="60">
-        <v>36573</v>
-      </c>
-      <c r="I17" s="11" t="str">
-        <v>Alaska Airlines</v>
-      </c>
-      <c r="J17" s="11" t="str">
-        <v>Viaggio d'affari</v>
-      </c>
-      <c r="K17" s="31">
-        <v>201000</v>
-      </c>
-      <c r="L17" s="11">
-        <v>14</v>
-      </c>
+      <c r="H17" s="72"/>
+      <c r="I17" s="31">
+        <v>183900</v>
+      </c>
+      <c r="K17" s="71"/>
+      <c r="L17" s="71"/>
       <c r="M17" s="9"/>
     </row>
     <row r="18" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34418,21 +34452,12 @@
       <c r="E18" s="26">
         <v>16</v>
       </c>
-      <c r="H18" s="60">
-        <v>36596</v>
-      </c>
-      <c r="I18" s="11" t="str">
-        <v>DAK Industries</v>
-      </c>
-      <c r="J18" s="11" t="str">
-        <v>Mobili</v>
-      </c>
-      <c r="K18" s="31">
+      <c r="H18" s="72"/>
+      <c r="I18" s="31">
         <v>183900</v>
       </c>
-      <c r="L18" s="11">
-        <v>26</v>
-      </c>
+      <c r="K18" s="71"/>
+      <c r="L18" s="71"/>
       <c r="M18" s="9"/>
     </row>
     <row r="19" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34451,21 +34476,12 @@
       <c r="E19" s="26">
         <v>13</v>
       </c>
-      <c r="H19" s="60">
-        <v>36637</v>
-      </c>
-      <c r="I19" s="11" t="str">
-        <v>DAK Industries</v>
-      </c>
-      <c r="J19" s="11" t="str">
-        <v>Mobili</v>
-      </c>
-      <c r="K19" s="31">
-        <v>183900</v>
-      </c>
-      <c r="L19" s="11">
-        <v>18</v>
-      </c>
+      <c r="H19" s="72"/>
+      <c r="I19" s="31">
+        <v>163500</v>
+      </c>
+      <c r="K19" s="71"/>
+      <c r="L19" s="71"/>
       <c r="M19" s="9"/>
     </row>
     <row r="20" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34484,21 +34500,12 @@
       <c r="E20" s="26">
         <v>20</v>
       </c>
-      <c r="H20" s="60">
-        <v>36596</v>
-      </c>
-      <c r="I20" s="11" t="str">
-        <v>After the Stork</v>
-      </c>
-      <c r="J20" s="11" t="str">
-        <v>Abbigliamento</v>
-      </c>
-      <c r="K20" s="31">
-        <v>163500</v>
-      </c>
-      <c r="L20" s="11">
-        <v>18</v>
-      </c>
+      <c r="H20" s="72"/>
+      <c r="I20" s="31">
+        <v>151500</v>
+      </c>
+      <c r="K20" s="71"/>
+      <c r="L20" s="71"/>
       <c r="M20" s="9"/>
     </row>
     <row r="21" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34517,21 +34524,12 @@
       <c r="E21" s="26">
         <v>18</v>
       </c>
-      <c r="H21" s="60">
-        <v>36580</v>
-      </c>
-      <c r="I21" s="11" t="str">
-        <v>Biobottoms</v>
-      </c>
-      <c r="J21" s="11" t="str">
-        <v>Abbigliamento</v>
-      </c>
-      <c r="K21" s="31">
-        <v>151500</v>
-      </c>
-      <c r="L21" s="11">
-        <v>13</v>
-      </c>
+      <c r="H21" s="72"/>
+      <c r="I21" s="31">
+        <v>127950</v>
+      </c>
+      <c r="K21" s="71"/>
+      <c r="L21" s="71"/>
       <c r="M21" s="9"/>
     </row>
     <row r="22" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34550,21 +34548,12 @@
       <c r="E22" s="26">
         <v>16</v>
       </c>
-      <c r="H22" s="60">
-        <v>36596</v>
-      </c>
-      <c r="I22" s="11" t="str">
-        <v>Avis</v>
-      </c>
-      <c r="J22" s="11" t="str">
-        <v>Viaggio d'affari: trasporto</v>
-      </c>
-      <c r="K22" s="31">
-        <v>127950</v>
-      </c>
-      <c r="L22" s="11">
-        <v>20</v>
-      </c>
+      <c r="H22" s="72"/>
+      <c r="I22" s="31">
+        <v>127490</v>
+      </c>
+      <c r="K22" s="71"/>
+      <c r="L22" s="71"/>
       <c r="M22" s="9"/>
     </row>
     <row r="23" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34583,21 +34572,12 @@
       <c r="E23" s="26">
         <v>14</v>
       </c>
-      <c r="H23" s="60">
-        <v>36558</v>
-      </c>
-      <c r="I23" s="11" t="str">
-        <v>Furrow Building Materials</v>
-      </c>
-      <c r="J23" s="11" t="str">
-        <v>Educazione dei figli</v>
-      </c>
-      <c r="K23" s="31">
+      <c r="H23" s="72"/>
+      <c r="I23" s="31">
         <v>127490</v>
       </c>
-      <c r="L23" s="11">
-        <v>17</v>
-      </c>
+      <c r="K23" s="71"/>
+      <c r="L23" s="71"/>
       <c r="M23" s="9"/>
     </row>
     <row r="24" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34616,21 +34596,12 @@
       <c r="E24" s="26">
         <v>14</v>
       </c>
-      <c r="H24" s="60">
-        <v>36598</v>
-      </c>
-      <c r="I24" s="11" t="str">
-        <v>Furrow Building Materials</v>
-      </c>
-      <c r="J24" s="11" t="str">
-        <v>Educazione dei figli</v>
-      </c>
-      <c r="K24" s="31">
-        <v>127490</v>
-      </c>
-      <c r="L24" s="11">
-        <v>21</v>
-      </c>
+      <c r="H24" s="72"/>
+      <c r="I24" s="31">
+        <v>98450</v>
+      </c>
+      <c r="K24" s="71"/>
+      <c r="L24" s="71"/>
       <c r="M24" s="9"/>
     </row>
     <row r="25" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34649,21 +34620,12 @@
       <c r="E25" s="26">
         <v>17</v>
       </c>
-      <c r="H25" s="60">
-        <v>36548</v>
-      </c>
-      <c r="I25" s="11" t="str">
-        <v>Canon USA</v>
-      </c>
-      <c r="J25" s="11" t="str">
-        <v>Ufficio</v>
-      </c>
-      <c r="K25" s="31">
-        <v>98450</v>
-      </c>
-      <c r="L25" s="11">
-        <v>21</v>
-      </c>
+      <c r="H25" s="72"/>
+      <c r="I25" s="31">
+        <v>87450</v>
+      </c>
+      <c r="K25" s="71"/>
+      <c r="L25" s="71"/>
       <c r="M25" s="9"/>
     </row>
     <row r="26" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34682,21 +34644,12 @@
       <c r="E26" s="26">
         <v>18</v>
       </c>
-      <c r="H26" s="60">
-        <v>36553</v>
-      </c>
-      <c r="I26" s="11" t="str">
-        <v>Deluxe Business Forms</v>
-      </c>
-      <c r="J26" s="11" t="str">
-        <v>Ufficio</v>
-      </c>
-      <c r="K26" s="31">
-        <v>87450</v>
-      </c>
-      <c r="L26" s="11">
-        <v>24</v>
-      </c>
+      <c r="H26" s="72"/>
+      <c r="I26" s="31">
+        <v>87300</v>
+      </c>
+      <c r="K26" s="71"/>
+      <c r="L26" s="71"/>
       <c r="M26" s="9"/>
     </row>
     <row r="27" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34715,21 +34668,12 @@
       <c r="E27" s="26">
         <v>14</v>
       </c>
-      <c r="H27" s="60">
-        <v>36603</v>
-      </c>
-      <c r="I27" s="11" t="str">
-        <v>Chinaberry Book</v>
-      </c>
-      <c r="J27" s="11" t="str">
-        <v>Svago</v>
-      </c>
-      <c r="K27" s="31">
-        <v>87300</v>
-      </c>
-      <c r="L27" s="11">
-        <v>18</v>
-      </c>
+      <c r="H27" s="72"/>
+      <c r="I27" s="31">
+        <v>84500</v>
+      </c>
+      <c r="K27" s="71"/>
+      <c r="L27" s="71"/>
       <c r="M27" s="9"/>
     </row>
     <row r="28" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34748,21 +34692,12 @@
       <c r="E28" s="26">
         <v>17</v>
       </c>
-      <c r="H28" s="60">
-        <v>36629</v>
-      </c>
-      <c r="I28" s="11" t="str">
-        <v>DeLorme Publishing</v>
-      </c>
-      <c r="J28" s="11" t="str">
-        <v>Software ufficio</v>
-      </c>
-      <c r="K28" s="31">
-        <v>84500</v>
-      </c>
-      <c r="L28" s="11">
-        <v>21</v>
-      </c>
+      <c r="H28" s="72"/>
+      <c r="I28" s="31">
+        <v>81500</v>
+      </c>
+      <c r="K28" s="71"/>
+      <c r="L28" s="71"/>
       <c r="M28" s="9"/>
     </row>
     <row r="29" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34781,21 +34716,12 @@
       <c r="E29" s="26">
         <v>18</v>
       </c>
-      <c r="H29" s="60">
-        <v>36637</v>
-      </c>
-      <c r="I29" s="11" t="str">
-        <v>Biobottoms</v>
-      </c>
-      <c r="J29" s="11" t="str">
-        <v>Abbigliamento</v>
-      </c>
-      <c r="K29" s="31">
-        <v>81500</v>
-      </c>
-      <c r="L29" s="11">
-        <v>25</v>
-      </c>
+      <c r="H29" s="72"/>
+      <c r="I29" s="31">
+        <v>78530</v>
+      </c>
+      <c r="K29" s="71"/>
+      <c r="L29" s="71"/>
       <c r="M29" s="9"/>
     </row>
     <row r="30" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34814,21 +34740,12 @@
       <c r="E30" s="26">
         <v>26</v>
       </c>
-      <c r="H30" s="60">
-        <v>36609</v>
-      </c>
-      <c r="I30" s="11" t="str">
-        <v>Avis</v>
-      </c>
-      <c r="J30" s="11" t="str">
-        <v>Viaggio d'affari: trasporto</v>
-      </c>
-      <c r="K30" s="31">
-        <v>78530</v>
-      </c>
-      <c r="L30" s="11">
-        <v>25</v>
-      </c>
+      <c r="H30" s="72"/>
+      <c r="I30" s="31">
+        <v>71800</v>
+      </c>
+      <c r="K30" s="71"/>
+      <c r="L30" s="71"/>
       <c r="M30" s="9"/>
     </row>
     <row r="31" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34847,21 +34764,12 @@
       <c r="E31" s="26">
         <v>16</v>
       </c>
-      <c r="H31" s="60">
-        <v>36595</v>
-      </c>
-      <c r="I31" s="11" t="str">
-        <v>Epcot Center</v>
-      </c>
-      <c r="J31" s="11" t="str">
-        <v>Svago</v>
-      </c>
-      <c r="K31" s="31">
-        <v>71800</v>
-      </c>
-      <c r="L31" s="11">
-        <v>18</v>
-      </c>
+      <c r="H31" s="72"/>
+      <c r="I31" s="31">
+        <v>55600</v>
+      </c>
+      <c r="K31" s="71"/>
+      <c r="L31" s="71"/>
       <c r="M31" s="9"/>
     </row>
     <row r="32" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34880,21 +34788,12 @@
       <c r="E32" s="26">
         <v>17</v>
       </c>
-      <c r="H32" s="60">
-        <v>36624</v>
-      </c>
-      <c r="I32" s="11" t="str">
-        <v>Elco Computers</v>
-      </c>
-      <c r="J32" s="11" t="str">
-        <v>Hardware</v>
-      </c>
-      <c r="K32" s="31">
-        <v>55600</v>
-      </c>
-      <c r="L32" s="11">
-        <v>11</v>
-      </c>
+      <c r="H32" s="72"/>
+      <c r="I32" s="31">
+        <v>51800</v>
+      </c>
+      <c r="K32" s="71"/>
+      <c r="L32" s="71"/>
       <c r="M32" s="9"/>
     </row>
     <row r="33" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34913,21 +34812,12 @@
       <c r="E33" s="26">
         <v>25</v>
       </c>
-      <c r="H33" s="60">
-        <v>36632</v>
-      </c>
-      <c r="I33" s="11" t="str">
-        <v>After the Stork</v>
-      </c>
-      <c r="J33" s="11" t="str">
-        <v>Abbigliamento</v>
-      </c>
-      <c r="K33" s="31">
-        <v>51800</v>
-      </c>
-      <c r="L33" s="11">
-        <v>21</v>
-      </c>
+      <c r="H33" s="72"/>
+      <c r="I33" s="31">
+        <v>50800</v>
+      </c>
+      <c r="K33" s="71"/>
+      <c r="L33" s="71"/>
       <c r="M33" s="9"/>
     </row>
     <row r="34" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34946,21 +34836,12 @@
       <c r="E34" s="26">
         <v>20</v>
       </c>
-      <c r="H34" s="60">
-        <v>36547</v>
-      </c>
-      <c r="I34" s="11" t="str">
-        <v>Allstate</v>
-      </c>
-      <c r="J34" s="11" t="str">
-        <v>Assicurazione</v>
-      </c>
-      <c r="K34" s="31">
-        <v>50800</v>
-      </c>
-      <c r="L34" s="11">
-        <v>22</v>
-      </c>
+      <c r="H34" s="72"/>
+      <c r="I34" s="31">
+        <v>50280</v>
+      </c>
+      <c r="K34" s="71"/>
+      <c r="L34" s="71"/>
       <c r="M34" s="9"/>
     </row>
     <row r="35" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -34979,21 +34860,12 @@
       <c r="E35" s="26">
         <v>23</v>
       </c>
-      <c r="H35" s="60">
-        <v>36700</v>
-      </c>
-      <c r="I35" s="11" t="str">
-        <v>H &amp; B Recordings</v>
-      </c>
-      <c r="J35" s="11" t="str">
-        <v>Svago</v>
-      </c>
-      <c r="K35" s="31">
-        <v>50280</v>
-      </c>
-      <c r="L35" s="11">
-        <v>20</v>
-      </c>
+      <c r="H35" s="72"/>
+      <c r="I35" s="31">
+        <v>50000</v>
+      </c>
+      <c r="K35" s="71"/>
+      <c r="L35" s="71"/>
       <c r="M35" s="9"/>
     </row>
     <row r="36" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35012,21 +34884,12 @@
       <c r="E36" s="26">
         <v>25</v>
       </c>
-      <c r="H36" s="60">
-        <v>36529</v>
-      </c>
-      <c r="I36" s="11" t="str">
-        <v>Ferguson and Bardell</v>
-      </c>
-      <c r="J36" s="11" t="str">
-        <v>Abbigliamento</v>
-      </c>
-      <c r="K36" s="31">
+      <c r="H36" s="72"/>
+      <c r="I36" s="31">
         <v>50000</v>
       </c>
-      <c r="L36" s="11">
-        <v>16</v>
-      </c>
+      <c r="K36" s="71"/>
+      <c r="L36" s="71"/>
       <c r="M36" s="9"/>
     </row>
     <row r="37" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35045,21 +34908,12 @@
       <c r="E37" s="26">
         <v>21</v>
       </c>
-      <c r="H37" s="60">
-        <v>36598</v>
-      </c>
-      <c r="I37" s="11" t="str">
-        <v>Ferguson and Bardell</v>
-      </c>
-      <c r="J37" s="11" t="str">
-        <v>Salute</v>
-      </c>
-      <c r="K37" s="31">
-        <v>50000</v>
-      </c>
-      <c r="L37" s="11">
-        <v>15</v>
-      </c>
+      <c r="H37" s="72"/>
+      <c r="I37" s="31">
+        <v>49400</v>
+      </c>
+      <c r="K37" s="71"/>
+      <c r="L37" s="71"/>
       <c r="M37" s="9"/>
     </row>
     <row r="38" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35078,21 +34932,12 @@
       <c r="E38" s="26">
         <v>17</v>
       </c>
-      <c r="H38" s="60">
-        <v>36558</v>
-      </c>
-      <c r="I38" s="11" t="str">
-        <v>Chinaberry Book</v>
-      </c>
-      <c r="J38" s="11" t="str">
-        <v>Svago</v>
-      </c>
-      <c r="K38" s="31">
-        <v>49400</v>
-      </c>
-      <c r="L38" s="11">
-        <v>13</v>
-      </c>
+      <c r="H38" s="72"/>
+      <c r="I38" s="31">
+        <v>45890</v>
+      </c>
+      <c r="K38" s="71"/>
+      <c r="L38" s="71"/>
       <c r="M38" s="9"/>
     </row>
     <row r="39" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35111,21 +34956,12 @@
       <c r="E39" s="26">
         <v>15</v>
       </c>
-      <c r="H39" s="60">
-        <v>36551</v>
-      </c>
-      <c r="I39" s="11" t="str">
-        <v>H&amp;B</v>
-      </c>
-      <c r="J39" s="11" t="str">
-        <v>Svago</v>
-      </c>
-      <c r="K39" s="31">
-        <v>45890</v>
-      </c>
-      <c r="L39" s="11">
-        <v>18</v>
-      </c>
+      <c r="H39" s="72"/>
+      <c r="I39" s="31">
+        <v>44950</v>
+      </c>
+      <c r="K39" s="71"/>
+      <c r="L39" s="71"/>
       <c r="M39" s="9"/>
     </row>
     <row r="40" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35144,21 +34980,12 @@
       <c r="E40" s="26">
         <v>24</v>
       </c>
-      <c r="H40" s="60">
-        <v>36622</v>
-      </c>
-      <c r="I40" s="11" t="str">
-        <v>Gardeners Eden</v>
-      </c>
-      <c r="J40" s="11" t="str">
-        <v>Abitazione</v>
-      </c>
-      <c r="K40" s="31">
-        <v>44950</v>
-      </c>
-      <c r="L40" s="11">
-        <v>20</v>
-      </c>
+      <c r="H40" s="72"/>
+      <c r="I40" s="31">
+        <v>43500</v>
+      </c>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
       <c r="M40" s="9"/>
     </row>
     <row r="41" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35177,21 +35004,12 @@
       <c r="E41" s="26">
         <v>18</v>
       </c>
-      <c r="H41" s="60">
-        <v>36543</v>
-      </c>
-      <c r="I41" s="11" t="str">
-        <v>Fletcher's for Children</v>
-      </c>
-      <c r="J41" s="11" t="str">
-        <v>Attrezzatura</v>
-      </c>
-      <c r="K41" s="31">
+      <c r="H41" s="72"/>
+      <c r="I41" s="31">
         <v>43500</v>
       </c>
-      <c r="L41" s="11">
-        <v>29</v>
-      </c>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
       <c r="M41" s="9"/>
     </row>
     <row r="42" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35210,21 +35028,12 @@
       <c r="E42" s="26">
         <v>11</v>
       </c>
-      <c r="H42" s="60">
-        <v>36596</v>
-      </c>
-      <c r="I42" s="11" t="str">
-        <v>Chambers</v>
-      </c>
-      <c r="J42" s="11" t="str">
-        <v>Regali</v>
-      </c>
-      <c r="K42" s="31">
-        <v>43500</v>
-      </c>
-      <c r="L42" s="11">
-        <v>16</v>
-      </c>
+      <c r="H42" s="72"/>
+      <c r="I42" s="31">
+        <v>40650</v>
+      </c>
+      <c r="K42" s="71"/>
+      <c r="L42" s="71"/>
       <c r="M42" s="9"/>
     </row>
     <row r="43" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35243,21 +35052,11 @@
       <c r="E43" s="26">
         <v>21</v>
       </c>
-      <c r="H43" s="60">
-        <v>36697</v>
-      </c>
-      <c r="I43" s="11" t="str">
-        <v>Bridgewater Restaurant, Florence</v>
-      </c>
-      <c r="J43" s="11" t="str">
-        <v>Ristorante</v>
-      </c>
-      <c r="K43" s="31">
-        <v>40650</v>
-      </c>
-      <c r="L43" s="11">
-        <v>17</v>
-      </c>
+      <c r="H43" s="72"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="71"/>
+      <c r="L43" s="71"/>
       <c r="M43" s="9"/>
     </row>
     <row r="44" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -35276,7 +35075,7 @@
       <c r="E44" s="26">
         <v>25</v>
       </c>
-      <c r="H44" s="48"/>
+      <c r="H44" s="47"/>
       <c r="I44" s="9"/>
       <c r="J44" s="9"/>
       <c r="K44" s="9"/>
@@ -35298,7 +35097,7 @@
       <c r="E45" s="26">
         <v>18</v>
       </c>
-      <c r="H45" s="48"/>
+      <c r="H45" s="47"/>
     </row>
     <row r="46" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="23">
@@ -35333,19 +35132,19 @@
       <c r="E47" s="26">
         <v>22</v>
       </c>
-      <c r="H47" s="65" t="s">
+      <c r="H47" s="60" t="s">
         <v>493</v>
       </c>
-      <c r="I47" s="66" t="s">
+      <c r="I47" s="61" t="s">
         <v>494</v>
       </c>
-      <c r="J47" s="66" t="s">
+      <c r="J47" s="61" t="s">
         <v>495</v>
       </c>
-      <c r="K47" s="66" t="s">
+      <c r="K47" s="61" t="s">
         <v>496</v>
       </c>
-      <c r="L47" s="67" t="s">
+      <c r="L47" s="62" t="s">
         <v>497</v>
       </c>
     </row>
@@ -35365,7 +35164,7 @@
       <c r="E48" s="26">
         <v>27</v>
       </c>
-      <c r="H48" s="61">
+      <c r="H48" s="58">
         <v>36604</v>
       </c>
       <c r="I48" s="11" t="s">
@@ -35377,7 +35176,7 @@
       <c r="K48" s="31">
         <v>2425000</v>
       </c>
-      <c r="L48" s="39">
+      <c r="L48" s="68">
         <v>11</v>
       </c>
     </row>
@@ -35397,7 +35196,7 @@
       <c r="E49" s="26">
         <v>18</v>
       </c>
-      <c r="H49" s="61">
+      <c r="H49" s="58">
         <v>36649</v>
       </c>
       <c r="I49" s="11" t="s">
@@ -35409,7 +35208,7 @@
       <c r="K49" s="31">
         <v>2425000</v>
       </c>
-      <c r="L49" s="39">
+      <c r="L49" s="68">
         <v>21</v>
       </c>
     </row>
@@ -35429,7 +35228,7 @@
       <c r="E50" s="26">
         <v>20</v>
       </c>
-      <c r="H50" s="61">
+      <c r="H50" s="58">
         <v>36651</v>
       </c>
       <c r="I50" s="11" t="s">
@@ -35441,7 +35240,7 @@
       <c r="K50" s="31">
         <v>1860000</v>
       </c>
-      <c r="L50" s="39">
+      <c r="L50" s="68">
         <v>19</v>
       </c>
     </row>
@@ -35461,7 +35260,7 @@
       <c r="E51" s="26">
         <v>11</v>
       </c>
-      <c r="H51" s="61">
+      <c r="H51" s="58">
         <v>36573</v>
       </c>
       <c r="I51" s="11" t="s">
@@ -35473,7 +35272,7 @@
       <c r="K51" s="31">
         <v>1368000</v>
       </c>
-      <c r="L51" s="39">
+      <c r="L51" s="68">
         <v>28</v>
       </c>
     </row>
@@ -35493,7 +35292,7 @@
       <c r="E52" s="26">
         <v>21</v>
       </c>
-      <c r="H52" s="61">
+      <c r="H52" s="58">
         <v>36555</v>
       </c>
       <c r="I52" s="11" t="s">
@@ -35505,7 +35304,7 @@
       <c r="K52" s="31">
         <v>348980</v>
       </c>
-      <c r="L52" s="39">
+      <c r="L52" s="68">
         <v>15</v>
       </c>
     </row>
@@ -35525,7 +35324,7 @@
       <c r="E53" s="26">
         <v>21</v>
       </c>
-      <c r="H53" s="61">
+      <c r="H53" s="58">
         <v>36554</v>
       </c>
       <c r="I53" s="11" t="s">
@@ -35537,7 +35336,7 @@
       <c r="K53" s="31">
         <v>295000</v>
       </c>
-      <c r="L53" s="39">
+      <c r="L53" s="68">
         <v>27</v>
       </c>
     </row>
@@ -35557,7 +35356,7 @@
       <c r="E54" s="26">
         <v>16</v>
       </c>
-      <c r="H54" s="61">
+      <c r="H54" s="58">
         <v>36573</v>
       </c>
       <c r="I54" s="11" t="s">
@@ -35569,7 +35368,7 @@
       <c r="K54" s="31">
         <v>201000</v>
       </c>
-      <c r="L54" s="39">
+      <c r="L54" s="68">
         <v>14</v>
       </c>
     </row>
@@ -35589,7 +35388,7 @@
       <c r="E55" s="26">
         <v>25</v>
       </c>
-      <c r="H55" s="61">
+      <c r="H55" s="58">
         <v>36596</v>
       </c>
       <c r="I55" s="11" t="s">
@@ -35601,7 +35400,7 @@
       <c r="K55" s="31">
         <v>183900</v>
       </c>
-      <c r="L55" s="39">
+      <c r="L55" s="68">
         <v>26</v>
       </c>
     </row>
@@ -35621,7 +35420,7 @@
       <c r="E56" s="26">
         <v>18</v>
       </c>
-      <c r="H56" s="61">
+      <c r="H56" s="58">
         <v>36637</v>
       </c>
       <c r="I56" s="11" t="s">
@@ -35633,7 +35432,7 @@
       <c r="K56" s="31">
         <v>183900</v>
       </c>
-      <c r="L56" s="39">
+      <c r="L56" s="68">
         <v>18</v>
       </c>
     </row>
@@ -35653,7 +35452,7 @@
       <c r="E57" s="26">
         <v>18</v>
       </c>
-      <c r="H57" s="61">
+      <c r="H57" s="58">
         <v>36596</v>
       </c>
       <c r="I57" s="11" t="s">
@@ -35665,7 +35464,7 @@
       <c r="K57" s="31">
         <v>163500</v>
       </c>
-      <c r="L57" s="39">
+      <c r="L57" s="68">
         <v>18</v>
       </c>
     </row>
@@ -35685,7 +35484,7 @@
       <c r="E58" s="26">
         <v>21</v>
       </c>
-      <c r="H58" s="61">
+      <c r="H58" s="58">
         <v>36580</v>
       </c>
       <c r="I58" s="11" t="s">
@@ -35697,7 +35496,7 @@
       <c r="K58" s="31">
         <v>151500</v>
       </c>
-      <c r="L58" s="39">
+      <c r="L58" s="68">
         <v>13</v>
       </c>
     </row>
@@ -35717,7 +35516,7 @@
       <c r="E59" s="26">
         <v>23</v>
       </c>
-      <c r="H59" s="61">
+      <c r="H59" s="58">
         <v>36596</v>
       </c>
       <c r="I59" s="11" t="s">
@@ -35729,7 +35528,7 @@
       <c r="K59" s="31">
         <v>127950</v>
       </c>
-      <c r="L59" s="39">
+      <c r="L59" s="68">
         <v>20</v>
       </c>
     </row>
@@ -35749,7 +35548,7 @@
       <c r="E60" s="26">
         <v>20</v>
       </c>
-      <c r="H60" s="61">
+      <c r="H60" s="58">
         <v>36558</v>
       </c>
       <c r="I60" s="11" t="s">
@@ -35761,7 +35560,7 @@
       <c r="K60" s="31">
         <v>127490</v>
       </c>
-      <c r="L60" s="39">
+      <c r="L60" s="68">
         <v>17</v>
       </c>
     </row>
@@ -35781,7 +35580,7 @@
       <c r="E61" s="26">
         <v>21</v>
       </c>
-      <c r="H61" s="61">
+      <c r="H61" s="58">
         <v>36598</v>
       </c>
       <c r="I61" s="11" t="s">
@@ -35793,7 +35592,7 @@
       <c r="K61" s="31">
         <v>127490</v>
       </c>
-      <c r="L61" s="39">
+      <c r="L61" s="68">
         <v>21</v>
       </c>
     </row>
@@ -35813,7 +35612,7 @@
       <c r="E62" s="26">
         <v>18</v>
       </c>
-      <c r="H62" s="61">
+      <c r="H62" s="58">
         <v>36548</v>
       </c>
       <c r="I62" s="11" t="s">
@@ -35825,7 +35624,7 @@
       <c r="K62" s="31">
         <v>98450</v>
       </c>
-      <c r="L62" s="39">
+      <c r="L62" s="68">
         <v>21</v>
       </c>
     </row>
@@ -35845,7 +35644,7 @@
       <c r="E63" s="26">
         <v>12</v>
       </c>
-      <c r="H63" s="61">
+      <c r="H63" s="58">
         <v>36553</v>
       </c>
       <c r="I63" s="11" t="s">
@@ -35857,7 +35656,7 @@
       <c r="K63" s="31">
         <v>87450</v>
       </c>
-      <c r="L63" s="39">
+      <c r="L63" s="68">
         <v>24</v>
       </c>
     </row>
@@ -35877,7 +35676,7 @@
       <c r="E64" s="26">
         <v>21</v>
       </c>
-      <c r="H64" s="61">
+      <c r="H64" s="58">
         <v>36603</v>
       </c>
       <c r="I64" s="11" t="s">
@@ -35889,7 +35688,7 @@
       <c r="K64" s="31">
         <v>87300</v>
       </c>
-      <c r="L64" s="39">
+      <c r="L64" s="68">
         <v>18</v>
       </c>
     </row>
@@ -35909,7 +35708,7 @@
       <c r="E65" s="26">
         <v>19</v>
       </c>
-      <c r="H65" s="61">
+      <c r="H65" s="58">
         <v>36629</v>
       </c>
       <c r="I65" s="11" t="s">
@@ -35921,7 +35720,7 @@
       <c r="K65" s="31">
         <v>84500</v>
       </c>
-      <c r="L65" s="39">
+      <c r="L65" s="68">
         <v>21</v>
       </c>
     </row>
@@ -35941,7 +35740,7 @@
       <c r="E66" s="26">
         <v>13</v>
       </c>
-      <c r="H66" s="61">
+      <c r="H66" s="58">
         <v>36637</v>
       </c>
       <c r="I66" s="11" t="s">
@@ -35953,7 +35752,7 @@
       <c r="K66" s="31">
         <v>81500</v>
       </c>
-      <c r="L66" s="39">
+      <c r="L66" s="68">
         <v>25</v>
       </c>
     </row>
@@ -35973,7 +35772,7 @@
       <c r="E67" s="26">
         <v>16</v>
       </c>
-      <c r="H67" s="61">
+      <c r="H67" s="58">
         <v>36609</v>
       </c>
       <c r="I67" s="11" t="s">
@@ -35985,7 +35784,7 @@
       <c r="K67" s="31">
         <v>78530</v>
       </c>
-      <c r="L67" s="39">
+      <c r="L67" s="68">
         <v>25</v>
       </c>
     </row>
@@ -36005,7 +35804,7 @@
       <c r="E68" s="26">
         <v>19</v>
       </c>
-      <c r="H68" s="61">
+      <c r="H68" s="58">
         <v>36595</v>
       </c>
       <c r="I68" s="11" t="s">
@@ -36017,7 +35816,7 @@
       <c r="K68" s="31">
         <v>71800</v>
       </c>
-      <c r="L68" s="39">
+      <c r="L68" s="68">
         <v>18</v>
       </c>
     </row>
@@ -36037,7 +35836,7 @@
       <c r="E69" s="26">
         <v>17</v>
       </c>
-      <c r="H69" s="61">
+      <c r="H69" s="58">
         <v>36624</v>
       </c>
       <c r="I69" s="11" t="s">
@@ -36049,7 +35848,7 @@
       <c r="K69" s="31">
         <v>55600</v>
       </c>
-      <c r="L69" s="39">
+      <c r="L69" s="68">
         <v>11</v>
       </c>
     </row>
@@ -36069,7 +35868,7 @@
       <c r="E70" s="26">
         <v>20</v>
       </c>
-      <c r="H70" s="61">
+      <c r="H70" s="58">
         <v>36632</v>
       </c>
       <c r="I70" s="11" t="s">
@@ -36081,7 +35880,7 @@
       <c r="K70" s="31">
         <v>51800</v>
       </c>
-      <c r="L70" s="39">
+      <c r="L70" s="68">
         <v>21</v>
       </c>
     </row>
@@ -36101,7 +35900,7 @@
       <c r="E71" s="26">
         <v>19</v>
       </c>
-      <c r="H71" s="61">
+      <c r="H71" s="58">
         <v>36547</v>
       </c>
       <c r="I71" s="11" t="s">
@@ -36113,7 +35912,7 @@
       <c r="K71" s="31">
         <v>50800</v>
       </c>
-      <c r="L71" s="39">
+      <c r="L71" s="68">
         <v>22</v>
       </c>
     </row>
@@ -36133,7 +35932,7 @@
       <c r="E72" s="26">
         <v>20</v>
       </c>
-      <c r="H72" s="61">
+      <c r="H72" s="58">
         <v>36700</v>
       </c>
       <c r="I72" s="11" t="s">
@@ -36145,7 +35944,7 @@
       <c r="K72" s="31">
         <v>50280</v>
       </c>
-      <c r="L72" s="39">
+      <c r="L72" s="68">
         <v>20</v>
       </c>
     </row>
@@ -36165,7 +35964,7 @@
       <c r="E73" s="26">
         <v>21</v>
       </c>
-      <c r="H73" s="61">
+      <c r="H73" s="58">
         <v>36529</v>
       </c>
       <c r="I73" s="11" t="s">
@@ -36177,7 +35976,7 @@
       <c r="K73" s="31">
         <v>50000</v>
       </c>
-      <c r="L73" s="39">
+      <c r="L73" s="68">
         <v>16</v>
       </c>
     </row>
@@ -36197,7 +35996,7 @@
       <c r="E74" s="26">
         <v>22</v>
       </c>
-      <c r="H74" s="61">
+      <c r="H74" s="58">
         <v>36598</v>
       </c>
       <c r="I74" s="11" t="s">
@@ -36209,7 +36008,7 @@
       <c r="K74" s="31">
         <v>50000</v>
       </c>
-      <c r="L74" s="39">
+      <c r="L74" s="68">
         <v>15</v>
       </c>
     </row>
@@ -36229,7 +36028,7 @@
       <c r="E75" s="26">
         <v>14</v>
       </c>
-      <c r="H75" s="61">
+      <c r="H75" s="58">
         <v>36558</v>
       </c>
       <c r="I75" s="11" t="s">
@@ -36241,7 +36040,7 @@
       <c r="K75" s="31">
         <v>49400</v>
       </c>
-      <c r="L75" s="39">
+      <c r="L75" s="68">
         <v>13</v>
       </c>
     </row>
@@ -36261,7 +36060,7 @@
       <c r="E76" s="26">
         <v>22</v>
       </c>
-      <c r="H76" s="61">
+      <c r="H76" s="58">
         <v>36551</v>
       </c>
       <c r="I76" s="11" t="s">
@@ -36273,7 +36072,7 @@
       <c r="K76" s="31">
         <v>45890</v>
       </c>
-      <c r="L76" s="39">
+      <c r="L76" s="68">
         <v>18</v>
       </c>
     </row>
@@ -36293,7 +36092,7 @@
       <c r="E77" s="26">
         <v>17</v>
       </c>
-      <c r="H77" s="61">
+      <c r="H77" s="58">
         <v>36622</v>
       </c>
       <c r="I77" s="11" t="s">
@@ -36305,7 +36104,7 @@
       <c r="K77" s="31">
         <v>44950</v>
       </c>
-      <c r="L77" s="39">
+      <c r="L77" s="68">
         <v>20</v>
       </c>
     </row>
@@ -36325,7 +36124,7 @@
       <c r="E78" s="26">
         <v>20</v>
       </c>
-      <c r="H78" s="61">
+      <c r="H78" s="58">
         <v>36543</v>
       </c>
       <c r="I78" s="11" t="s">
@@ -36337,7 +36136,7 @@
       <c r="K78" s="31">
         <v>43500</v>
       </c>
-      <c r="L78" s="39">
+      <c r="L78" s="68">
         <v>29</v>
       </c>
     </row>
@@ -36357,7 +36156,7 @@
       <c r="E79" s="26">
         <v>21</v>
       </c>
-      <c r="H79" s="61">
+      <c r="H79" s="58">
         <v>36596</v>
       </c>
       <c r="I79" s="11" t="s">
@@ -36369,7 +36168,7 @@
       <c r="K79" s="31">
         <v>43500</v>
       </c>
-      <c r="L79" s="39">
+      <c r="L79" s="68">
         <v>16</v>
       </c>
     </row>
@@ -36389,7 +36188,7 @@
       <c r="E80" s="30">
         <v>28</v>
       </c>
-      <c r="H80" s="62">
+      <c r="H80" s="59">
         <v>36697</v>
       </c>
       <c r="I80" s="12" t="s">
@@ -36398,81 +36197,100 @@
       <c r="J80" s="12" t="s">
         <v>524</v>
       </c>
-      <c r="K80" s="68">
+      <c r="K80" s="63">
         <v>40650</v>
       </c>
-      <c r="L80" s="42">
+      <c r="L80" s="69">
         <v>17</v>
       </c>
     </row>
-    <row r="81" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D81" s="7"/>
       <c r="E81" s="7"/>
-    </row>
-    <row r="82" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D82" s="7"/>
+      <c r="H81" s="74" t="s">
+        <v>712</v>
+      </c>
+      <c r="I81" s="12"/>
+      <c r="J81" s="12"/>
+      <c r="K81" s="75">
+        <f>SUBTOTAL(109,fatture40k[Importo fattura])</f>
+        <v>11154610</v>
+      </c>
+      <c r="L81" s="69">
+        <f>SUBTOTAL(109,fatture40k[Spese di spedizione])</f>
+        <v>638</v>
+      </c>
+    </row>
+    <row r="82" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C82" s="46" t="s">
+        <v>710</v>
+      </c>
+      <c r="D82" s="67">
+        <f>SUM(Importo_fattura)</f>
+        <v>11954160</v>
+      </c>
       <c r="E82" s="7"/>
     </row>
-    <row r="83" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
-      <c r="K83" s="71" t="s">
+    </row>
+    <row r="84" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D84" s="7"/>
+      <c r="E84" s="7"/>
+      <c r="K84" s="66" t="s">
         <v>709</v>
       </c>
-      <c r="L83" s="69">
+      <c r="L84" s="64">
         <f>SUM(fatture40k[Importo fattura])</f>
         <v>11154610</v>
       </c>
     </row>
-    <row r="84" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
-    </row>
-    <row r="85" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D85" s="7"/>
       <c r="E85" s="7"/>
     </row>
-    <row r="86" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D86" s="7"/>
       <c r="E86" s="7"/>
     </row>
-    <row r="87" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D87" s="7"/>
       <c r="E87" s="7"/>
     </row>
-    <row r="88" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D88" s="7"/>
       <c r="E88" s="7"/>
     </row>
-    <row r="89" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D89" s="7"/>
       <c r="E89" s="7"/>
     </row>
-    <row r="90" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D90" s="7"/>
       <c r="E90" s="7"/>
     </row>
-    <row r="91" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D91" s="7"/>
       <c r="E91" s="7"/>
     </row>
-    <row r="92" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D92" s="7"/>
       <c r="E92" s="7"/>
     </row>
-    <row r="93" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D93" s="7"/>
       <c r="E93" s="7"/>
     </row>
-    <row r="94" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D94" s="7"/>
       <c r="E94" s="7"/>
     </row>
-    <row r="95" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D95" s="7"/>
       <c r="E95" s="7"/>
     </row>
-    <row r="96" spans="4:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D96" s="7"/>
       <c r="E96" s="7"/>
     </row>
@@ -40979,7 +40797,7 @@
       <c r="F1" s="44" t="s">
         <v>706</v>
       </c>
-      <c r="G1" s="49" t="s">
+      <c r="G1" s="48" t="s">
         <v>703</v>
       </c>
       <c r="H1" s="46" t="s">
@@ -40993,20 +40811,20 @@
       <c r="B2" s="38">
         <v>55</v>
       </c>
-      <c r="C2" s="55">
+      <c r="C2" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>102.06919642857143</v>
       </c>
       <c r="D2" s="39"/>
-      <c r="E2" s="51" t="str">
+      <c r="E2" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F2" s="53">
+      <c r="F2" s="51">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
-      <c r="G2" s="50" t="str" cm="1">
+      <c r="G2" s="49" t="str" cm="1">
         <f t="array" ref="G2:G6">_xlfn.UNIQUE(frutta[FRUTTA])</f>
         <v>Mela</v>
       </c>
@@ -41022,22 +40840,22 @@
       <c r="B3" s="38">
         <v>70</v>
       </c>
-      <c r="C3" s="55">
+      <c r="C3" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>80</v>
       </c>
       <c r="D3" s="36">
         <v>80</v>
       </c>
-      <c r="E3" s="51">
+      <c r="E3" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.1428571428571428</v>
       </c>
-      <c r="F3" s="51">
+      <c r="F3" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
-      <c r="G3" s="50" t="str">
+      <c r="G3" s="49" t="str">
         <v>Banana</v>
       </c>
       <c r="H3" s="11">
@@ -41052,22 +40870,22 @@
       <c r="B4" s="38">
         <v>40</v>
       </c>
-      <c r="C4" s="55">
+      <c r="C4" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>60</v>
       </c>
       <c r="D4" s="36">
         <v>60</v>
       </c>
-      <c r="E4" s="51">
+      <c r="E4" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.5</v>
       </c>
-      <c r="F4" s="51">
+      <c r="F4" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
-      <c r="G4" s="50" t="str">
+      <c r="G4" s="49" t="str">
         <v>Arancia</v>
       </c>
       <c r="H4" s="11">
@@ -41082,22 +40900,22 @@
       <c r="B5" s="38">
         <v>20</v>
       </c>
-      <c r="C5" s="55">
+      <c r="C5" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>100</v>
       </c>
       <c r="D5" s="36">
         <v>100</v>
       </c>
-      <c r="E5" s="51">
+      <c r="E5" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>5</v>
       </c>
-      <c r="F5" s="51">
+      <c r="F5" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
-      <c r="G5" s="50" t="str">
+      <c r="G5" s="49" t="str">
         <v>Pera</v>
       </c>
       <c r="H5" s="11">
@@ -41112,22 +40930,22 @@
       <c r="B6" s="38">
         <v>90</v>
       </c>
-      <c r="C6" s="55">
+      <c r="C6" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>30</v>
       </c>
       <c r="D6" s="36">
         <v>30</v>
       </c>
-      <c r="E6" s="51">
+      <c r="E6" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F6" s="51">
+      <c r="F6" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
-      <c r="G6" s="50" t="str">
+      <c r="G6" s="49" t="str">
         <v>Uva</v>
       </c>
       <c r="H6" s="11">
@@ -41142,18 +40960,18 @@
       <c r="B7" s="38">
         <v>50</v>
       </c>
-      <c r="C7" s="55">
+      <c r="C7" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>40</v>
       </c>
       <c r="D7" s="36">
         <v>40</v>
       </c>
-      <c r="E7" s="52">
+      <c r="E7" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.8</v>
       </c>
-      <c r="F7" s="52">
+      <c r="F7" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41165,18 +40983,18 @@
       <c r="B8" s="38">
         <v>60</v>
       </c>
-      <c r="C8" s="55">
+      <c r="C8" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>55</v>
       </c>
       <c r="D8" s="36">
         <v>55</v>
       </c>
-      <c r="E8" s="52">
+      <c r="E8" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.91666666666666663</v>
       </c>
-      <c r="F8" s="52">
+      <c r="F8" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41188,16 +41006,16 @@
       <c r="B9" s="38">
         <v>45</v>
       </c>
-      <c r="C9" s="55">
+      <c r="C9" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>83.511160714285708</v>
       </c>
       <c r="D9" s="39"/>
-      <c r="E9" s="52" t="str">
+      <c r="E9" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41209,18 +41027,18 @@
       <c r="B10" s="38">
         <v>25</v>
       </c>
-      <c r="C10" s="55">
+      <c r="C10" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>85</v>
       </c>
       <c r="D10" s="36">
         <v>85</v>
       </c>
-      <c r="E10" s="52">
+      <c r="E10" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>3.4</v>
       </c>
-      <c r="F10" s="52">
+      <c r="F10" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41232,18 +41050,18 @@
       <c r="B11" s="38">
         <v>35</v>
       </c>
-      <c r="C11" s="55">
+      <c r="C11" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>50</v>
       </c>
       <c r="D11" s="36">
         <v>50</v>
       </c>
-      <c r="E11" s="52">
+      <c r="E11" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="F11" s="52">
+      <c r="F11" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -41255,18 +41073,18 @@
       <c r="B12" s="38">
         <v>60</v>
       </c>
-      <c r="C12" s="55">
+      <c r="C12" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>95</v>
       </c>
       <c r="D12" s="36">
         <v>95</v>
       </c>
-      <c r="E12" s="52">
+      <c r="E12" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.5833333333333333</v>
       </c>
-      <c r="F12" s="52">
+      <c r="F12" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.9959207459207458</v>
       </c>
@@ -41278,16 +41096,16 @@
       <c r="B13" s="38">
         <v>80</v>
       </c>
-      <c r="C13" s="55">
+      <c r="C13" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>100.49523809523811</v>
       </c>
       <c r="D13" s="39"/>
-      <c r="E13" s="52" t="str">
+      <c r="E13" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F13" s="52">
+      <c r="F13" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41299,18 +41117,18 @@
       <c r="B14" s="38">
         <v>40</v>
       </c>
-      <c r="C14" s="55">
+      <c r="C14" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>45</v>
       </c>
       <c r="D14" s="36">
         <v>45</v>
       </c>
-      <c r="E14" s="52">
+      <c r="E14" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.125</v>
       </c>
-      <c r="F14" s="52">
+      <c r="F14" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41322,18 +41140,18 @@
       <c r="B15" s="38">
         <v>65</v>
       </c>
-      <c r="C15" s="55">
+      <c r="C15" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>65</v>
       </c>
       <c r="D15" s="36">
         <v>65</v>
       </c>
-      <c r="E15" s="52">
+      <c r="E15" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1</v>
       </c>
-      <c r="F15" s="52">
+      <c r="F15" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41345,18 +41163,18 @@
       <c r="B16" s="38">
         <v>55</v>
       </c>
-      <c r="C16" s="55">
+      <c r="C16" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>30</v>
       </c>
       <c r="D16" s="36">
         <v>30</v>
       </c>
-      <c r="E16" s="52">
+      <c r="E16" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.54545454545454541</v>
       </c>
-      <c r="F16" s="52">
+      <c r="F16" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41368,16 +41186,16 @@
       <c r="B17" s="38">
         <v>70</v>
       </c>
-      <c r="C17" s="55">
+      <c r="C17" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>91.71875</v>
       </c>
       <c r="D17" s="39"/>
-      <c r="E17" s="52" t="str">
+      <c r="E17" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F17" s="52">
+      <c r="F17" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -41389,18 +41207,18 @@
       <c r="B18" s="38">
         <v>45</v>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>80</v>
       </c>
       <c r="D18" s="36">
         <v>80</v>
       </c>
-      <c r="E18" s="52">
+      <c r="E18" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.7777777777777777</v>
       </c>
-      <c r="F18" s="52">
+      <c r="F18" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41412,18 +41230,18 @@
       <c r="B19" s="38">
         <v>25</v>
       </c>
-      <c r="C19" s="55">
+      <c r="C19" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>60</v>
       </c>
       <c r="D19" s="36">
         <v>60</v>
       </c>
-      <c r="E19" s="52">
+      <c r="E19" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>2.4</v>
       </c>
-      <c r="F19" s="52">
+      <c r="F19" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41435,16 +41253,16 @@
       <c r="B20" s="38">
         <v>35</v>
       </c>
-      <c r="C20" s="55">
+      <c r="C20" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>48.746527777777771</v>
       </c>
       <c r="D20" s="39"/>
-      <c r="E20" s="52" t="str">
+      <c r="E20" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F20" s="52">
+      <c r="F20" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41456,18 +41274,18 @@
       <c r="B21" s="38">
         <v>60</v>
       </c>
-      <c r="C21" s="55">
+      <c r="C21" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>30</v>
       </c>
       <c r="D21" s="36">
         <v>30</v>
       </c>
-      <c r="E21" s="52">
+      <c r="E21" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.5</v>
       </c>
-      <c r="F21" s="52">
+      <c r="F21" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41479,18 +41297,18 @@
       <c r="B22" s="38">
         <v>70</v>
       </c>
-      <c r="C22" s="55">
+      <c r="C22" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>40</v>
       </c>
       <c r="D22" s="36">
         <v>40</v>
       </c>
-      <c r="E22" s="52">
+      <c r="E22" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.5714285714285714</v>
       </c>
-      <c r="F22" s="52">
+      <c r="F22" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41502,18 +41320,18 @@
       <c r="B23" s="38">
         <v>45</v>
       </c>
-      <c r="C23" s="55">
+      <c r="C23" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>55</v>
       </c>
       <c r="D23" s="36">
         <v>55</v>
       </c>
-      <c r="E23" s="52">
+      <c r="E23" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.2222222222222223</v>
       </c>
-      <c r="F23" s="52">
+      <c r="F23" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41525,18 +41343,18 @@
       <c r="B24" s="38">
         <v>25</v>
       </c>
-      <c r="C24" s="55">
+      <c r="C24" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>70</v>
       </c>
       <c r="D24" s="36">
         <v>70</v>
       </c>
-      <c r="E24" s="52">
+      <c r="E24" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>2.8</v>
       </c>
-      <c r="F24" s="52">
+      <c r="F24" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -41548,16 +41366,16 @@
       <c r="B25" s="38">
         <v>35</v>
       </c>
-      <c r="C25" s="55">
+      <c r="C25" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>69.857226107226097</v>
       </c>
       <c r="D25" s="39"/>
-      <c r="E25" s="52" t="str">
+      <c r="E25" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F25" s="52">
+      <c r="F25" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.9959207459207458</v>
       </c>
@@ -41569,18 +41387,18 @@
       <c r="B26" s="38">
         <v>60</v>
       </c>
-      <c r="C26" s="55">
+      <c r="C26" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>50</v>
       </c>
       <c r="D26" s="36">
         <v>50</v>
       </c>
-      <c r="E26" s="52">
+      <c r="E26" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.83333333333333337</v>
       </c>
-      <c r="F26" s="52">
+      <c r="F26" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41592,18 +41410,18 @@
       <c r="B27" s="38">
         <v>80</v>
       </c>
-      <c r="C27" s="55">
+      <c r="C27" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>95</v>
       </c>
       <c r="D27" s="36">
         <v>95</v>
       </c>
-      <c r="E27" s="52">
+      <c r="E27" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.1875</v>
       </c>
-      <c r="F27" s="52">
+      <c r="F27" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41615,18 +41433,18 @@
       <c r="B28" s="38">
         <v>40</v>
       </c>
-      <c r="C28" s="55">
+      <c r="C28" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>75</v>
       </c>
       <c r="D28" s="36">
         <v>75</v>
       </c>
-      <c r="E28" s="52">
+      <c r="E28" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.875</v>
       </c>
-      <c r="F28" s="52">
+      <c r="F28" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41638,18 +41456,18 @@
       <c r="B29" s="38">
         <v>65</v>
       </c>
-      <c r="C29" s="55">
+      <c r="C29" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>45</v>
       </c>
       <c r="D29" s="36">
         <v>45</v>
       </c>
-      <c r="E29" s="52">
+      <c r="E29" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.69230769230769229</v>
       </c>
-      <c r="F29" s="52">
+      <c r="F29" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41661,18 +41479,18 @@
       <c r="B30" s="38">
         <v>55</v>
       </c>
-      <c r="C30" s="55">
+      <c r="C30" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>65</v>
       </c>
       <c r="D30" s="36">
         <v>65</v>
       </c>
-      <c r="E30" s="52">
+      <c r="E30" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.1818181818181819</v>
       </c>
-      <c r="F30" s="52">
+      <c r="F30" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41684,18 +41502,18 @@
       <c r="B31" s="38">
         <v>70</v>
       </c>
-      <c r="C31" s="55">
+      <c r="C31" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>30</v>
       </c>
       <c r="D31" s="36">
         <v>30</v>
       </c>
-      <c r="E31" s="52">
+      <c r="E31" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.42857142857142855</v>
       </c>
-      <c r="F31" s="52">
+      <c r="F31" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -41707,16 +41525,16 @@
       <c r="B32" s="38">
         <v>45</v>
       </c>
-      <c r="C32" s="55">
+      <c r="C32" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>83.511160714285708</v>
       </c>
       <c r="D32" s="39"/>
-      <c r="E32" s="52" t="str">
+      <c r="E32" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F32" s="52">
+      <c r="F32" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41728,18 +41546,18 @@
       <c r="B33" s="38">
         <v>25</v>
       </c>
-      <c r="C33" s="55">
+      <c r="C33" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>80</v>
       </c>
       <c r="D33" s="36">
         <v>80</v>
       </c>
-      <c r="E33" s="52">
+      <c r="E33" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>3.2</v>
       </c>
-      <c r="F33" s="52">
+      <c r="F33" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41751,18 +41569,18 @@
       <c r="B34" s="38">
         <v>35</v>
       </c>
-      <c r="C34" s="55">
+      <c r="C34" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>60</v>
       </c>
       <c r="D34" s="36">
         <v>60</v>
       </c>
-      <c r="E34" s="52">
+      <c r="E34" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.7142857142857142</v>
       </c>
-      <c r="F34" s="52">
+      <c r="F34" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41774,18 +41592,18 @@
       <c r="B35" s="38">
         <v>60</v>
       </c>
-      <c r="C35" s="55">
+      <c r="C35" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>100</v>
       </c>
       <c r="D35" s="36">
         <v>100</v>
       </c>
-      <c r="E35" s="52">
+      <c r="E35" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.6666666666666667</v>
       </c>
-      <c r="F35" s="52">
+      <c r="F35" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41797,18 +41615,18 @@
       <c r="B36" s="38">
         <v>80</v>
       </c>
-      <c r="C36" s="55">
+      <c r="C36" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>30</v>
       </c>
       <c r="D36" s="36">
         <v>30</v>
       </c>
-      <c r="E36" s="52">
+      <c r="E36" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.375</v>
       </c>
-      <c r="F36" s="52">
+      <c r="F36" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41820,16 +41638,16 @@
       <c r="B37" s="38">
         <v>40</v>
       </c>
-      <c r="C37" s="55">
+      <c r="C37" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>52.410714285714292</v>
       </c>
       <c r="D37" s="39"/>
-      <c r="E37" s="52" t="str">
+      <c r="E37" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F37" s="52">
+      <c r="F37" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -41841,18 +41659,18 @@
       <c r="B38" s="38">
         <v>65</v>
       </c>
-      <c r="C38" s="55">
+      <c r="C38" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>55</v>
       </c>
       <c r="D38" s="36">
         <v>55</v>
       </c>
-      <c r="E38" s="52">
+      <c r="E38" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.84615384615384615</v>
       </c>
-      <c r="F38" s="52">
+      <c r="F38" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.9959207459207458</v>
       </c>
@@ -41864,18 +41682,18 @@
       <c r="B39" s="38">
         <v>55</v>
       </c>
-      <c r="C39" s="55">
+      <c r="C39" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>70</v>
       </c>
       <c r="D39" s="36">
         <v>70</v>
       </c>
-      <c r="E39" s="52">
+      <c r="E39" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.2727272727272727</v>
       </c>
-      <c r="F39" s="52">
+      <c r="F39" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41887,18 +41705,18 @@
       <c r="B40" s="38">
         <v>70</v>
       </c>
-      <c r="C40" s="55">
+      <c r="C40" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>85</v>
       </c>
       <c r="D40" s="36">
         <v>85</v>
       </c>
-      <c r="E40" s="52">
+      <c r="E40" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.2142857142857142</v>
       </c>
-      <c r="F40" s="52">
+      <c r="F40" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41910,18 +41728,18 @@
       <c r="B41" s="38">
         <v>40</v>
       </c>
-      <c r="C41" s="55">
+      <c r="C41" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>50</v>
       </c>
       <c r="D41" s="36">
         <v>50</v>
       </c>
-      <c r="E41" s="52">
+      <c r="E41" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.25</v>
       </c>
-      <c r="F41" s="52">
+      <c r="F41" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -41933,18 +41751,18 @@
       <c r="B42" s="38">
         <v>20</v>
       </c>
-      <c r="C42" s="55">
+      <c r="C42" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>95</v>
       </c>
       <c r="D42" s="36">
         <v>95</v>
       </c>
-      <c r="E42" s="52">
+      <c r="E42" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>4.75</v>
       </c>
-      <c r="F42" s="52">
+      <c r="F42" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>
@@ -41956,18 +41774,18 @@
       <c r="B43" s="38">
         <v>90</v>
       </c>
-      <c r="C43" s="55">
+      <c r="C43" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>75</v>
       </c>
       <c r="D43" s="36">
         <v>75</v>
       </c>
-      <c r="E43" s="52">
+      <c r="E43" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.83333333333333337</v>
       </c>
-      <c r="F43" s="52">
+      <c r="F43" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -41979,18 +41797,18 @@
       <c r="B44" s="38">
         <v>50</v>
       </c>
-      <c r="C44" s="55">
+      <c r="C44" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>45</v>
       </c>
       <c r="D44" s="36">
         <v>45</v>
       </c>
-      <c r="E44" s="52">
+      <c r="E44" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>0.9</v>
       </c>
-      <c r="F44" s="52">
+      <c r="F44" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3102678571428572</v>
       </c>
@@ -42002,18 +41820,18 @@
       <c r="B45" s="38">
         <v>60</v>
       </c>
-      <c r="C45" s="55">
+      <c r="C45" s="53">
         <f>IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>65</v>
       </c>
       <c r="D45" s="36">
         <v>65</v>
       </c>
-      <c r="E45" s="52">
+      <c r="E45" s="50">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v>1.0833333333333333</v>
       </c>
-      <c r="F45" s="52">
+      <c r="F45" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.8558035714285714</v>
       </c>
@@ -42025,16 +41843,16 @@
       <c r="B46" s="38">
         <v>45</v>
       </c>
-      <c r="C46" s="55">
+      <c r="C46" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>62.674107142857132</v>
       </c>
       <c r="D46" s="39"/>
-      <c r="E46" s="52" t="str">
+      <c r="E46" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F46" s="52">
+      <c r="F46" s="50">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.3927579365079363</v>
       </c>
@@ -42046,16 +41864,16 @@
       <c r="B47" s="41">
         <v>25</v>
       </c>
-      <c r="C47" s="55">
+      <c r="C47" s="53">
         <f ca="1">IF(frutta[[#This Row],[COSTO]]="",frutta[[#This Row],[PESO]]*frutta[[#This Row],[PREZZO UNITARIO MEDIO ]],frutta[[#This Row],[COSTO]])</f>
         <v>31.404761904761909</v>
       </c>
       <c r="D47" s="42"/>
-      <c r="E47" s="52" t="str">
+      <c r="E47" s="50" t="str">
         <f>IF(frutta[[#This Row],[COSTO]]="","",frutta[[#This Row],[COSTO]]/frutta[[#This Row],[PESO]])</f>
         <v/>
       </c>
-      <c r="F47" s="54">
+      <c r="F47" s="52">
         <f ca="1">_xlfn.XLOOKUP(frutta[[#This Row],[FRUTTA]],$G$2:$G$6,$H$2:$H$6)</f>
         <v>1.2561904761904763</v>
       </c>

</xml_diff>